<commit_message>
Update final data karyawan
</commit_message>
<xml_diff>
--- a/SSJ - Prime Database TAD.xlsx
+++ b/SSJ - Prime Database TAD.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30327"/>
-  <workbookPr codeName="ThisWorkbook"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\Dropbox\1.2 SSJ\HRIS SYSTEM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\Dropbox\1.2 SSJ\HRIS SYSTEM\hris-donggi-matindok\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4ADB407E-ABFC-4E41-AC70-CF704D88B9B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA67E4EA-5E95-4D14-B0A9-E6657AD01CFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" tabRatio="1000" xr2:uid="{29D13372-D5E9-4BA4-A471-6BF912524645}"/>
   </bookViews>
@@ -2939,17 +2939,17 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="9">
-    <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="165" formatCode="yyyy"/>
-    <numFmt numFmtId="166" formatCode="[$-13809]d\ mmm\ yyyy;@"/>
-    <numFmt numFmtId="167" formatCode="0\ &quot;Day(s)&quot;"/>
-    <numFmt numFmtId="168" formatCode="yy\ &quot;Years(s)&quot;\,\ mm\ &quot;Month(s)&quot;\,\ dd\ &quot;Day(s)&quot;"/>
-    <numFmt numFmtId="169" formatCode="yy\ &quot;Tahun&quot;\,\ mm\ &quot;Bulan&quot;\,\ dd\ &quot;Hari&quot;"/>
-    <numFmt numFmtId="170" formatCode="@* &quot;:&quot;"/>
-    <numFmt numFmtId="171" formatCode="[$-13809]dd\ mmmm\ yyyy;@"/>
-    <numFmt numFmtId="172" formatCode="_-[$Rp-421]* #,##0.00_-;\-[$Rp-421]* #,##0.00_-;_-[$Rp-421]* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="yyyy"/>
+    <numFmt numFmtId="165" formatCode="[$-13809]d\ mmm\ yyyy;@"/>
+    <numFmt numFmtId="166" formatCode="0\ &quot;Day(s)&quot;"/>
+    <numFmt numFmtId="167" formatCode="yy\ &quot;Years(s)&quot;\,\ mm\ &quot;Month(s)&quot;\,\ dd\ &quot;Day(s)&quot;"/>
+    <numFmt numFmtId="168" formatCode="yy\ &quot;Tahun&quot;\,\ mm\ &quot;Bulan&quot;\,\ dd\ &quot;Hari&quot;"/>
+    <numFmt numFmtId="169" formatCode="@* &quot;:&quot;"/>
+    <numFmt numFmtId="170" formatCode="[$-13809]dd\ mmmm\ yyyy;@"/>
+    <numFmt numFmtId="171" formatCode="_-[$Rp-421]* #,##0.00_-;\-[$Rp-421]* #,##0.00_-;_-[$Rp-421]* &quot;-&quot;_-;_-@_-"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3169,7 +3169,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -3180,7 +3180,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="12" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -3219,8 +3219,8 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="170" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="171" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="169" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="170" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -3239,7 +3239,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="172" fontId="10" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="171" fontId="10" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -3247,38 +3247,38 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="1" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="1" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="1" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="1" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="1" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="1" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3297,7 +3297,7 @@
     <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="169" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -3306,10 +3306,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="1" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="1" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="172" fontId="1" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="171" fontId="1" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -3681,83 +3681,83 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6FA82A2-3DDB-4E38-B511-C93A67A57491}">
   <sheetPr codeName="Sheet5"/>
   <dimension ref="A1:BU61"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" outlineLevelRow="1" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="12.75" outlineLevelRow="1" outlineLevelCol="1" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="7.7109375" style="3" customWidth="1"/>
-    <col min="2" max="2" width="10.140625" style="2" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="3" max="3" width="13.85546875" style="2" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="4" max="4" width="16.7109375" style="3" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="5" max="5" width="16.7109375" style="2" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="6" max="6" width="26.140625" style="2" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="1" max="1" width="7.73046875" style="3" customWidth="1"/>
+    <col min="2" max="2" width="10.1328125" style="2" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="3" max="3" width="13.86328125" style="2" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="4" max="4" width="16.73046875" style="3" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="5" max="5" width="16.73046875" style="2" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="6" max="6" width="26.1328125" style="2" bestFit="1" customWidth="1" collapsed="1"/>
     <col min="7" max="7" width="26" style="2" customWidth="1"/>
-    <col min="8" max="8" width="16.140625" style="2" customWidth="1" outlineLevel="1"/>
-    <col min="9" max="9" width="17.85546875" style="2" customWidth="1" outlineLevel="1"/>
-    <col min="10" max="10" width="9.85546875" style="2" customWidth="1"/>
-    <col min="11" max="11" width="12.7109375" style="3" customWidth="1" outlineLevel="1"/>
+    <col min="8" max="8" width="16.1328125" style="2" customWidth="1" outlineLevel="1"/>
+    <col min="9" max="9" width="17.86328125" style="2" customWidth="1" outlineLevel="1"/>
+    <col min="10" max="10" width="9.86328125" style="2" customWidth="1"/>
+    <col min="11" max="11" width="12.73046875" style="3" customWidth="1" outlineLevel="1"/>
     <col min="12" max="12" width="19" style="2" customWidth="1" outlineLevel="1"/>
-    <col min="13" max="13" width="31.140625" style="2" customWidth="1" outlineLevel="1"/>
-    <col min="14" max="14" width="10.28515625" style="2" customWidth="1"/>
-    <col min="15" max="15" width="17.85546875" style="2" customWidth="1" outlineLevel="1" collapsed="1"/>
-    <col min="16" max="16" width="17.28515625" style="3" customWidth="1" outlineLevel="1"/>
-    <col min="17" max="17" width="12.42578125" style="2" customWidth="1" outlineLevel="1" collapsed="1"/>
-    <col min="18" max="18" width="4.85546875" style="2" customWidth="1"/>
-    <col min="19" max="19" width="24.42578125" style="2" customWidth="1" outlineLevel="1"/>
-    <col min="20" max="20" width="25.7109375" style="2" customWidth="1"/>
-    <col min="21" max="21" width="13.42578125" style="2" customWidth="1" outlineLevel="1"/>
-    <col min="22" max="22" width="10.7109375" style="3" customWidth="1" outlineLevel="1"/>
+    <col min="13" max="13" width="31.1328125" style="2" customWidth="1" outlineLevel="1"/>
+    <col min="14" max="14" width="10.265625" style="2" customWidth="1"/>
+    <col min="15" max="15" width="17.86328125" style="2" customWidth="1" outlineLevel="1" collapsed="1"/>
+    <col min="16" max="16" width="17.265625" style="3" customWidth="1" outlineLevel="1"/>
+    <col min="17" max="17" width="12.3984375" style="2" customWidth="1" outlineLevel="1" collapsed="1"/>
+    <col min="18" max="18" width="4.86328125" style="2" customWidth="1"/>
+    <col min="19" max="19" width="24.3984375" style="2" customWidth="1" outlineLevel="1"/>
+    <col min="20" max="20" width="25.73046875" style="2" customWidth="1"/>
+    <col min="21" max="21" width="13.3984375" style="2" customWidth="1" outlineLevel="1"/>
+    <col min="22" max="22" width="10.73046875" style="3" customWidth="1" outlineLevel="1"/>
     <col min="23" max="23" width="16" style="2" customWidth="1" outlineLevel="1"/>
     <col min="24" max="24" width="10" style="2" customWidth="1" outlineLevel="1"/>
     <col min="25" max="25" width="9" style="2" customWidth="1"/>
-    <col min="26" max="26" width="18.140625" style="2" customWidth="1" outlineLevel="1"/>
-    <col min="27" max="27" width="38.42578125" style="2" customWidth="1" outlineLevel="1"/>
-    <col min="28" max="28" width="46.85546875" style="2" customWidth="1" outlineLevel="1"/>
-    <col min="29" max="29" width="6.42578125" style="3" customWidth="1" outlineLevel="1"/>
-    <col min="30" max="30" width="18.85546875" style="3" customWidth="1" outlineLevel="1"/>
-    <col min="31" max="31" width="14.140625" style="2" customWidth="1" outlineLevel="1" collapsed="1"/>
-    <col min="32" max="32" width="19.42578125" style="2" customWidth="1" outlineLevel="1"/>
+    <col min="26" max="26" width="18.1328125" style="2" customWidth="1" outlineLevel="1"/>
+    <col min="27" max="27" width="38.3984375" style="2" customWidth="1" outlineLevel="1"/>
+    <col min="28" max="28" width="46.86328125" style="2" customWidth="1" outlineLevel="1"/>
+    <col min="29" max="29" width="6.3984375" style="3" customWidth="1" outlineLevel="1"/>
+    <col min="30" max="30" width="18.86328125" style="3" customWidth="1" outlineLevel="1"/>
+    <col min="31" max="31" width="14.1328125" style="2" customWidth="1" outlineLevel="1" collapsed="1"/>
+    <col min="32" max="32" width="19.3984375" style="2" customWidth="1" outlineLevel="1"/>
     <col min="33" max="33" width="13" style="2" customWidth="1" outlineLevel="1"/>
     <col min="34" max="34" width="16" style="2" customWidth="1" outlineLevel="1" collapsed="1"/>
-    <col min="35" max="35" width="12.7109375" style="2" customWidth="1" outlineLevel="1" collapsed="1"/>
-    <col min="36" max="36" width="12.7109375" style="2" customWidth="1"/>
-    <col min="37" max="37" width="13.42578125" style="2" customWidth="1"/>
-    <col min="38" max="38" width="13.28515625" style="3" customWidth="1" outlineLevel="1"/>
-    <col min="39" max="39" width="10.42578125" style="2" customWidth="1" outlineLevel="1"/>
-    <col min="40" max="40" width="9.85546875" style="2" customWidth="1" outlineLevel="1"/>
-    <col min="41" max="41" width="34.28515625" style="2" customWidth="1" outlineLevel="1"/>
-    <col min="42" max="42" width="22.28515625" style="2" customWidth="1" outlineLevel="1"/>
-    <col min="43" max="43" width="13.42578125" style="2" customWidth="1" outlineLevel="1"/>
-    <col min="44" max="44" width="14.28515625" style="2" customWidth="1" outlineLevel="1"/>
+    <col min="35" max="35" width="12.73046875" style="2" customWidth="1" outlineLevel="1" collapsed="1"/>
+    <col min="36" max="36" width="12.73046875" style="2" customWidth="1"/>
+    <col min="37" max="37" width="13.3984375" style="2" customWidth="1"/>
+    <col min="38" max="38" width="13.265625" style="3" customWidth="1" outlineLevel="1"/>
+    <col min="39" max="39" width="10.3984375" style="2" customWidth="1" outlineLevel="1"/>
+    <col min="40" max="40" width="9.86328125" style="2" customWidth="1" outlineLevel="1"/>
+    <col min="41" max="41" width="34.265625" style="2" customWidth="1" outlineLevel="1"/>
+    <col min="42" max="42" width="22.265625" style="2" customWidth="1" outlineLevel="1"/>
+    <col min="43" max="43" width="13.3984375" style="2" customWidth="1" outlineLevel="1"/>
+    <col min="44" max="44" width="14.265625" style="2" customWidth="1" outlineLevel="1"/>
     <col min="45" max="45" width="12" style="2" customWidth="1" outlineLevel="1"/>
-    <col min="46" max="46" width="19.7109375" style="2" customWidth="1" outlineLevel="1"/>
-    <col min="47" max="47" width="17.28515625" style="3" customWidth="1" outlineLevel="1"/>
+    <col min="46" max="46" width="19.73046875" style="2" customWidth="1" outlineLevel="1"/>
+    <col min="47" max="47" width="17.265625" style="3" customWidth="1" outlineLevel="1"/>
     <col min="48" max="48" width="16" style="2" customWidth="1" outlineLevel="1" collapsed="1"/>
-    <col min="49" max="49" width="7.42578125" style="2" customWidth="1"/>
-    <col min="50" max="50" width="11.42578125" style="2" customWidth="1"/>
-    <col min="51" max="51" width="7.140625" style="2" customWidth="1" outlineLevel="1"/>
-    <col min="52" max="52" width="15.7109375" style="2" customWidth="1"/>
+    <col min="49" max="49" width="7.3984375" style="2" customWidth="1"/>
+    <col min="50" max="50" width="11.3984375" style="2" customWidth="1"/>
+    <col min="51" max="51" width="7.1328125" style="2" customWidth="1" outlineLevel="1"/>
+    <col min="52" max="52" width="15.73046875" style="2" customWidth="1"/>
     <col min="53" max="53" width="33" style="2" customWidth="1" outlineLevel="1"/>
-    <col min="54" max="54" width="35.85546875" style="2" customWidth="1" outlineLevel="1" collapsed="1"/>
-    <col min="55" max="55" width="57.85546875" style="2" customWidth="1" outlineLevel="1"/>
-    <col min="56" max="56" width="13.7109375" style="2" customWidth="1" outlineLevel="1"/>
-    <col min="57" max="57" width="8.140625" style="2" customWidth="1" outlineLevel="1"/>
-    <col min="58" max="58" width="15.85546875" style="2" customWidth="1" outlineLevel="1"/>
-    <col min="59" max="59" width="9.28515625" style="2" customWidth="1" outlineLevel="1"/>
+    <col min="54" max="54" width="35.86328125" style="2" customWidth="1" outlineLevel="1" collapsed="1"/>
+    <col min="55" max="55" width="57.86328125" style="2" customWidth="1" outlineLevel="1"/>
+    <col min="56" max="56" width="13.73046875" style="2" customWidth="1" outlineLevel="1"/>
+    <col min="57" max="57" width="8.1328125" style="2" customWidth="1" outlineLevel="1"/>
+    <col min="58" max="58" width="15.86328125" style="2" customWidth="1" outlineLevel="1"/>
+    <col min="59" max="59" width="9.265625" style="2" customWidth="1" outlineLevel="1"/>
     <col min="60" max="60" width="17" style="2" customWidth="1" outlineLevel="1"/>
     <col min="61" max="61" width="17" style="3" customWidth="1" outlineLevel="1"/>
-    <col min="62" max="62" width="15.140625" style="3" customWidth="1" outlineLevel="1"/>
-    <col min="63" max="63" width="12.85546875" style="3" customWidth="1" outlineLevel="1"/>
+    <col min="62" max="62" width="15.1328125" style="3" customWidth="1" outlineLevel="1"/>
+    <col min="63" max="63" width="12.86328125" style="3" customWidth="1" outlineLevel="1"/>
     <col min="64" max="64" width="17" style="2" customWidth="1" outlineLevel="1" collapsed="1"/>
-    <col min="65" max="65" width="22.42578125" style="2" customWidth="1" outlineLevel="1"/>
-    <col min="66" max="66" width="15.42578125" style="2" customWidth="1" outlineLevel="1"/>
+    <col min="65" max="65" width="22.3984375" style="2" customWidth="1" outlineLevel="1"/>
+    <col min="66" max="66" width="15.3984375" style="2" customWidth="1" outlineLevel="1"/>
     <col min="67" max="67" width="15" style="2" customWidth="1"/>
-    <col min="68" max="68" width="13.42578125" style="2" customWidth="1"/>
-    <col min="69" max="70" width="9.7109375" style="2" customWidth="1" outlineLevel="1"/>
+    <col min="68" max="68" width="13.3984375" style="2" customWidth="1"/>
+    <col min="69" max="70" width="9.73046875" style="2" customWidth="1" outlineLevel="1"/>
     <col min="71" max="71" width="6" style="3" customWidth="1"/>
-    <col min="72" max="72" width="18.85546875" style="3" customWidth="1"/>
-    <col min="73" max="16384" width="9.140625" style="3"/>
+    <col min="72" max="72" width="18.86328125" style="3" customWidth="1"/>
+    <col min="73" max="16384" width="9.1328125" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:73" ht="20.65">
+    <row r="1" spans="1:73" ht="20.65" x14ac:dyDescent="0.6">
       <c r="A1" s="53" t="s">
         <v>0</v>
       </c>
@@ -3834,7 +3834,7 @@
       <c r="BT1" s="44"/>
       <c r="BU1" s="44"/>
     </row>
-    <row r="3" spans="1:73" ht="13.15">
+    <row r="3" spans="1:73" ht="13.15" x14ac:dyDescent="0.4">
       <c r="A3" s="17" t="s">
         <v>1</v>
       </c>
@@ -3844,7 +3844,7 @@
       <c r="E3" s="52"/>
       <c r="F3" s="18">
         <f ca="1">TODAY()</f>
-        <v>46237</v>
+        <v>46238</v>
       </c>
       <c r="G3" s="52"/>
       <c r="H3" s="52"/>
@@ -3919,7 +3919,7 @@
       <c r="BT3" s="44"/>
       <c r="BU3" s="44"/>
     </row>
-    <row r="4" spans="1:73" ht="13.15">
+    <row r="4" spans="1:73" ht="13.15" x14ac:dyDescent="0.4">
       <c r="A4" s="17" t="s">
         <v>3</v>
       </c>
@@ -4003,7 +4003,7 @@
       <c r="BT4" s="44"/>
       <c r="BU4" s="44"/>
     </row>
-    <row r="5" spans="1:73" s="2" customFormat="1" outlineLevel="1">
+    <row r="5" spans="1:73" s="2" customFormat="1" outlineLevel="1" x14ac:dyDescent="0.35">
       <c r="A5" s="48">
         <v>1</v>
       </c>
@@ -4012,7 +4012,7 @@
         <v>0</v>
       </c>
       <c r="C5" s="48">
-        <f t="shared" ref="C5:BR5" si="0">COUNTBLANK(C7:C58)</f>
+        <f t="shared" ref="C5:E5" si="0">COUNTBLANK(C7:C58)</f>
         <v>0</v>
       </c>
       <c r="D5" s="48">
@@ -4290,7 +4290,7 @@
       </c>
       <c r="BU5" s="52"/>
     </row>
-    <row r="6" spans="1:73" s="16" customFormat="1" ht="32.25" customHeight="1">
+    <row r="6" spans="1:73" s="16" customFormat="1" ht="32.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="15" t="s">
         <v>5</v>
       </c>
@@ -4507,7 +4507,7 @@
       </c>
       <c r="BU6" s="21"/>
     </row>
-    <row r="7" spans="1:73" ht="14.25">
+    <row r="7" spans="1:73" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A7" s="26">
         <v>1</v>
       </c>
@@ -4565,11 +4565,11 @@
       </c>
       <c r="S7" s="31" t="str">
         <f ca="1">DATEDIF(Q7,TODAY(),"Y")&amp;" Tahun "&amp;DATEDIF(Q7,TODAY(),"YM")&amp;" Bulan "&amp;DATEDIF(Q7,TODAY(),"MD")&amp;" Hari "</f>
-        <v xml:space="preserve">34 Tahun 7 Bulan 9 Hari </v>
+        <v xml:space="preserve">34 Tahun 7 Bulan 10 Hari </v>
       </c>
       <c r="T7" s="32">
         <f t="shared" ref="T7:T58" ca="1" si="3">DATE(YEAR(Q7)+56,MONTH(Q7),DAY(Q7))-TODAY()</f>
-        <v>7814</v>
+        <v>7813</v>
       </c>
       <c r="U7" s="30" t="str">
         <f t="shared" ref="U7:U58" ca="1" si="4">IF(OR(R7="-",R7=""),"",IF(R7&lt;20,"&lt; 20 Tahun",IF(R7&lt;=25,"21-25 Tahun",IF(R7&lt;=30,"26-30 Tahun",IF(R7&lt;=35,"31-35 Tahun",IF(R7&lt;=40,"36-40 Tahun",IF(R7&lt;=45,"41-45 Tahun",IF(R7&lt;=50,"46-50 Tahun",IF(R7&lt;=55,"51-55 Tahun","56 Tahun Keatas")))))))))</f>
@@ -4623,7 +4623,7 @@
       </c>
       <c r="AK7" s="34">
         <f ca="1">AJ7-TODAY()+1</f>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL7" s="4">
         <v>41640</v>
@@ -4717,7 +4717,7 @@
       </c>
       <c r="BP7" s="34">
         <f ca="1">(BO7+365)-TODAY()+1</f>
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="BQ7" s="10" t="s">
         <v>120</v>
@@ -4731,7 +4731,7 @@
       </c>
       <c r="BU7" s="44"/>
     </row>
-    <row r="8" spans="1:73" ht="14.25">
+    <row r="8" spans="1:73" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A8" s="26">
         <v>2</v>
       </c>
@@ -4789,11 +4789,11 @@
       </c>
       <c r="S8" s="31" t="str">
         <f t="shared" ref="S8:S58" ca="1" si="7">DATEDIF(Q8,TODAY(),"Y")&amp;" Tahun "&amp;DATEDIF(Q8,TODAY(),"YM")&amp;" Bulan "&amp;DATEDIF(Q8,TODAY(),"MD")&amp;" Hari "</f>
-        <v xml:space="preserve">35 Tahun 2 Bulan 15 Hari </v>
+        <v xml:space="preserve">35 Tahun 2 Bulan 16 Hari </v>
       </c>
       <c r="T8" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>7594</v>
+        <v>7593</v>
       </c>
       <c r="U8" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -4848,7 +4848,7 @@
       </c>
       <c r="AK8" s="34">
         <f t="shared" ref="AK8:AK58" ca="1" si="8">AJ8-TODAY()+1</f>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL8" s="4">
         <v>41640</v>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="BP8" s="34">
         <f ca="1">(BO8+365)-TODAY()+1</f>
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="BQ8" s="10" t="s">
         <v>120</v>
@@ -4958,7 +4958,7 @@
       </c>
       <c r="BU8" s="44"/>
     </row>
-    <row r="9" spans="1:73" ht="14.25">
+    <row r="9" spans="1:73" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A9" s="26">
         <v>3</v>
       </c>
@@ -5016,11 +5016,11 @@
       </c>
       <c r="S9" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">49 Tahun 6 Bulan 16 Hari </v>
+        <v xml:space="preserve">49 Tahun 6 Bulan 17 Hari </v>
       </c>
       <c r="T9" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>2360</v>
+        <v>2359</v>
       </c>
       <c r="U9" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -5075,7 +5075,7 @@
       </c>
       <c r="AK9" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL9" s="4">
         <v>41640</v>
@@ -5169,7 +5169,7 @@
       </c>
       <c r="BP9" s="34">
         <f ca="1">(BO9+365)-TODAY()+1</f>
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="BQ9" s="10" t="s">
         <v>120</v>
@@ -5183,7 +5183,7 @@
       </c>
       <c r="BU9" s="44"/>
     </row>
-    <row r="10" spans="1:73" ht="14.25">
+    <row r="10" spans="1:73" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A10" s="26">
         <v>4</v>
       </c>
@@ -5241,11 +5241,11 @@
       </c>
       <c r="S10" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">28 Tahun 1 Bulan 24 Hari </v>
+        <v xml:space="preserve">28 Tahun 1 Bulan 25 Hari </v>
       </c>
       <c r="T10" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>10173</v>
+        <v>10172</v>
       </c>
       <c r="U10" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -5300,7 +5300,7 @@
       </c>
       <c r="AK10" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL10" s="4">
         <v>41640</v>
@@ -5394,7 +5394,7 @@
       </c>
       <c r="BP10" s="34">
         <f ca="1">(BO10+365)-TODAY()+1</f>
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="BQ10" s="10" t="s">
         <v>120</v>
@@ -5408,7 +5408,7 @@
       </c>
       <c r="BU10" s="44"/>
     </row>
-    <row r="11" spans="1:73" ht="14.25">
+    <row r="11" spans="1:73" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A11" s="26">
         <v>5</v>
       </c>
@@ -5466,11 +5466,11 @@
       </c>
       <c r="S11" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">41 Tahun 6 Bulan 2 Hari </v>
+        <v xml:space="preserve">41 Tahun 6 Bulan 3 Hari </v>
       </c>
       <c r="T11" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>5296</v>
+        <v>5295</v>
       </c>
       <c r="U11" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -5525,7 +5525,7 @@
       </c>
       <c r="AK11" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL11" s="4">
         <v>41640</v>
@@ -5619,7 +5619,7 @@
       </c>
       <c r="BP11" s="34">
         <f ca="1">(BO11+365)-TODAY()+1</f>
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="BQ11" s="10" t="s">
         <v>120</v>
@@ -5633,7 +5633,7 @@
       </c>
       <c r="BU11" s="44"/>
     </row>
-    <row r="12" spans="1:73" ht="14.25">
+    <row r="12" spans="1:73" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A12" s="26">
         <v>6</v>
       </c>
@@ -5691,11 +5691,11 @@
       </c>
       <c r="S12" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">33 Tahun 9 Bulan 2 Hari </v>
+        <v xml:space="preserve">33 Tahun 9 Bulan 3 Hari </v>
       </c>
       <c r="T12" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>8126</v>
+        <v>8125</v>
       </c>
       <c r="U12" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -5750,7 +5750,7 @@
       </c>
       <c r="AK12" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL12" s="4">
         <v>41640</v>
@@ -5846,7 +5846,7 @@
       </c>
       <c r="BP12" s="34">
         <f t="shared" ref="BP12:BP58" ca="1" si="10">(BO12+365)-TODAY()+1</f>
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="BQ12" s="10" t="s">
         <v>120</v>
@@ -5860,7 +5860,7 @@
       </c>
       <c r="BU12" s="44"/>
     </row>
-    <row r="13" spans="1:73" ht="14.25">
+    <row r="13" spans="1:73" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A13" s="26">
         <v>7</v>
       </c>
@@ -5918,11 +5918,11 @@
       </c>
       <c r="S13" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">42 Tahun 5 Bulan 1 Hari </v>
+        <v xml:space="preserve">42 Tahun 5 Bulan 2 Hari </v>
       </c>
       <c r="T13" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>4960</v>
+        <v>4959</v>
       </c>
       <c r="U13" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -5977,7 +5977,7 @@
       </c>
       <c r="AK13" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL13" s="4">
         <v>41640</v>
@@ -6071,7 +6071,7 @@
       </c>
       <c r="BP13" s="34">
         <f t="shared" ca="1" si="10"/>
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="BQ13" s="10" t="s">
         <v>120</v>
@@ -6085,7 +6085,7 @@
       </c>
       <c r="BU13" s="44"/>
     </row>
-    <row r="14" spans="1:73" ht="14.25">
+    <row r="14" spans="1:73" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A14" s="26">
         <v>8</v>
       </c>
@@ -6143,11 +6143,11 @@
       </c>
       <c r="S14" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">30 Tahun 6 Bulan 1 Hari </v>
+        <v xml:space="preserve">30 Tahun 6 Bulan 2 Hari </v>
       </c>
       <c r="T14" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>9314</v>
+        <v>9313</v>
       </c>
       <c r="U14" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -6202,7 +6202,7 @@
       </c>
       <c r="AK14" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL14" s="4">
         <v>41640</v>
@@ -6298,7 +6298,7 @@
       </c>
       <c r="BP14" s="34">
         <f t="shared" ca="1" si="10"/>
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="BQ14" s="10" t="s">
         <v>120</v>
@@ -6312,7 +6312,7 @@
       </c>
       <c r="BU14" s="44"/>
     </row>
-    <row r="15" spans="1:73" ht="14.25">
+    <row r="15" spans="1:73" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A15" s="26">
         <v>9</v>
       </c>
@@ -6368,11 +6368,11 @@
       </c>
       <c r="S15" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">36 Tahun 10 Bulan 0 Hari </v>
+        <v xml:space="preserve">36 Tahun 10 Bulan 1 Hari </v>
       </c>
       <c r="T15" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>7001</v>
+        <v>7000</v>
       </c>
       <c r="U15" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -6427,7 +6427,7 @@
       </c>
       <c r="AK15" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL15" s="4">
         <v>45880</v>
@@ -6522,7 +6522,7 @@
       </c>
       <c r="BP15" s="34">
         <f t="shared" ca="1" si="10"/>
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="BQ15" s="10" t="s">
         <v>120</v>
@@ -6536,7 +6536,7 @@
       </c>
       <c r="BU15" s="44"/>
     </row>
-    <row r="16" spans="1:73" ht="14.25">
+    <row r="16" spans="1:73" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A16" s="26">
         <v>10</v>
       </c>
@@ -6594,11 +6594,11 @@
       </c>
       <c r="S16" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">32 Tahun 2 Bulan 8 Hari </v>
+        <v xml:space="preserve">32 Tahun 2 Bulan 9 Hari </v>
       </c>
       <c r="T16" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>8697</v>
+        <v>8696</v>
       </c>
       <c r="U16" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -6653,7 +6653,7 @@
       </c>
       <c r="AK16" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL16" s="4">
         <v>41640</v>
@@ -6749,7 +6749,7 @@
       </c>
       <c r="BP16" s="34">
         <f t="shared" ca="1" si="10"/>
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="BQ16" s="10" t="s">
         <v>120</v>
@@ -6763,7 +6763,7 @@
       </c>
       <c r="BU16" s="44"/>
     </row>
-    <row r="17" spans="1:72" ht="14.25">
+    <row r="17" spans="1:72" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A17" s="26">
         <v>11</v>
       </c>
@@ -6821,11 +6821,11 @@
       </c>
       <c r="S17" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">22 Tahun 9 Bulan 4 Hari </v>
+        <v xml:space="preserve">22 Tahun 9 Bulan 5 Hari </v>
       </c>
       <c r="T17" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>12141</v>
+        <v>12140</v>
       </c>
       <c r="U17" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -6880,7 +6880,7 @@
       </c>
       <c r="AK17" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL17" s="4">
         <v>41640</v>
@@ -6974,7 +6974,7 @@
       </c>
       <c r="BP17" s="34">
         <f t="shared" ca="1" si="10"/>
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="BQ17" s="10" t="s">
         <v>120</v>
@@ -6987,7 +6987,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="18" spans="1:72" ht="14.25">
+    <row r="18" spans="1:72" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A18" s="26">
         <v>12</v>
       </c>
@@ -7043,11 +7043,11 @@
       </c>
       <c r="S18" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">26 Tahun 4 Bulan 22 Hari </v>
+        <v xml:space="preserve">26 Tahun 4 Bulan 23 Hari </v>
       </c>
       <c r="T18" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>10814</v>
+        <v>10813</v>
       </c>
       <c r="U18" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -7102,7 +7102,7 @@
       </c>
       <c r="AK18" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL18" s="4">
         <v>45880</v>
@@ -7195,7 +7195,7 @@
       </c>
       <c r="BP18" s="34">
         <f t="shared" ca="1" si="10"/>
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="BQ18" s="10" t="s">
         <v>120</v>
@@ -7208,7 +7208,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="19" spans="1:72" ht="14.25">
+    <row r="19" spans="1:72" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A19" s="26">
         <v>13</v>
       </c>
@@ -7266,11 +7266,11 @@
       </c>
       <c r="S19" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">48 Tahun 4 Bulan 22 Hari </v>
+        <v xml:space="preserve">48 Tahun 4 Bulan 23 Hari </v>
       </c>
       <c r="T19" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>2778</v>
+        <v>2777</v>
       </c>
       <c r="U19" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -7325,7 +7325,7 @@
       </c>
       <c r="AK19" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL19" s="4">
         <v>41640</v>
@@ -7419,7 +7419,7 @@
       </c>
       <c r="BP19" s="34">
         <f t="shared" ca="1" si="10"/>
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="BQ19" s="10" t="s">
         <v>120</v>
@@ -7432,7 +7432,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="20" spans="1:72" ht="14.25">
+    <row r="20" spans="1:72" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A20" s="26">
         <v>14</v>
       </c>
@@ -7490,11 +7490,11 @@
       </c>
       <c r="S20" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">40 Tahun 3 Bulan 17 Hari </v>
+        <v xml:space="preserve">40 Tahun 3 Bulan 18 Hari </v>
       </c>
       <c r="T20" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>5736</v>
+        <v>5735</v>
       </c>
       <c r="U20" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -7549,7 +7549,7 @@
       </c>
       <c r="AK20" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL20" s="4">
         <v>41640</v>
@@ -7643,7 +7643,7 @@
       </c>
       <c r="BP20" s="34">
         <f t="shared" ca="1" si="10"/>
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="BQ20" s="10" t="s">
         <v>120</v>
@@ -7656,7 +7656,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="21" spans="1:72" ht="14.25">
+    <row r="21" spans="1:72" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A21" s="26">
         <v>15</v>
       </c>
@@ -7714,11 +7714,11 @@
       </c>
       <c r="S21" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">32 Tahun 4 Bulan 17 Hari </v>
+        <v xml:space="preserve">32 Tahun 4 Bulan 18 Hari </v>
       </c>
       <c r="T21" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>8627</v>
+        <v>8626</v>
       </c>
       <c r="U21" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -7773,7 +7773,7 @@
       </c>
       <c r="AK21" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL21" s="4">
         <v>41640</v>
@@ -7869,7 +7869,7 @@
       </c>
       <c r="BP21" s="34">
         <f t="shared" ca="1" si="10"/>
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="BQ21" s="10" t="s">
         <v>120</v>
@@ -7882,7 +7882,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="22" spans="1:72" ht="14.25">
+    <row r="22" spans="1:72" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A22" s="26">
         <v>16</v>
       </c>
@@ -7940,11 +7940,11 @@
       </c>
       <c r="S22" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">42 Tahun 8 Bulan 29 Hari </v>
+        <v xml:space="preserve">42 Tahun 8 Bulan 30 Hari </v>
       </c>
       <c r="T22" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>4842</v>
+        <v>4841</v>
       </c>
       <c r="U22" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -7999,7 +7999,7 @@
       </c>
       <c r="AK22" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL22" s="4">
         <v>41640</v>
@@ -8093,7 +8093,7 @@
       </c>
       <c r="BP22" s="34">
         <f t="shared" ca="1" si="10"/>
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="BQ22" s="10" t="s">
         <v>120</v>
@@ -8106,7 +8106,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="23" spans="1:72" ht="14.25">
+    <row r="23" spans="1:72" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A23" s="26">
         <v>17</v>
       </c>
@@ -8164,11 +8164,11 @@
       </c>
       <c r="S23" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">31 Tahun 6 Bulan 30 Hari </v>
+        <v xml:space="preserve">31 Tahun 7 Bulan 0 Hari </v>
       </c>
       <c r="T23" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>8920</v>
+        <v>8919</v>
       </c>
       <c r="U23" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -8223,7 +8223,7 @@
       </c>
       <c r="AK23" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL23" s="4">
         <v>41640</v>
@@ -8319,7 +8319,7 @@
       </c>
       <c r="BP23" s="34">
         <f t="shared" ca="1" si="10"/>
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="BQ23" s="10" t="s">
         <v>120</v>
@@ -8332,7 +8332,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="24" spans="1:72" ht="14.25">
+    <row r="24" spans="1:72" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A24" s="26">
         <v>18</v>
       </c>
@@ -8390,11 +8390,11 @@
       </c>
       <c r="S24" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">50 Tahun 6 Bulan 2 Hari </v>
+        <v xml:space="preserve">50 Tahun 6 Bulan 3 Hari </v>
       </c>
       <c r="T24" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>2008</v>
+        <v>2007</v>
       </c>
       <c r="U24" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -8449,7 +8449,7 @@
       </c>
       <c r="AK24" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL24" s="4">
         <v>41640</v>
@@ -8545,7 +8545,7 @@
       </c>
       <c r="BP24" s="34">
         <f t="shared" ca="1" si="10"/>
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="BQ24" s="10" t="s">
         <v>120</v>
@@ -8558,7 +8558,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="25" spans="1:72" ht="14.25">
+    <row r="25" spans="1:72" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A25" s="26">
         <v>19</v>
       </c>
@@ -8614,11 +8614,11 @@
       </c>
       <c r="S25" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">28 Tahun 6 Bulan 16 Hari </v>
+        <v xml:space="preserve">28 Tahun 6 Bulan 17 Hari </v>
       </c>
       <c r="T25" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>10030</v>
+        <v>10029</v>
       </c>
       <c r="U25" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -8673,7 +8673,7 @@
       </c>
       <c r="AK25" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL25" s="35">
         <v>45800</v>
@@ -8767,7 +8767,7 @@
       </c>
       <c r="BP25" s="34">
         <f t="shared" ca="1" si="10"/>
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="BQ25" s="10" t="s">
         <v>120</v>
@@ -8780,7 +8780,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="26" spans="1:72" ht="14.25">
+    <row r="26" spans="1:72" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A26" s="26">
         <v>20</v>
       </c>
@@ -8838,11 +8838,11 @@
       </c>
       <c r="S26" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">46 Tahun 1 Bulan 30 Hari </v>
+        <v xml:space="preserve">46 Tahun 2 Bulan 0 Hari </v>
       </c>
       <c r="T26" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>3593</v>
+        <v>3592</v>
       </c>
       <c r="U26" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -8897,7 +8897,7 @@
       </c>
       <c r="AK26" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL26" s="4">
         <v>41640</v>
@@ -8991,7 +8991,7 @@
       </c>
       <c r="BP26" s="34">
         <f t="shared" ca="1" si="10"/>
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="BQ26" s="10" t="s">
         <v>120</v>
@@ -9004,7 +9004,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="27" spans="1:72" ht="14.25">
+    <row r="27" spans="1:72" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A27" s="26">
         <v>21</v>
       </c>
@@ -9062,11 +9062,11 @@
       </c>
       <c r="S27" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">48 Tahun 3 Bulan 24 Hari </v>
+        <v xml:space="preserve">48 Tahun 3 Bulan 25 Hari </v>
       </c>
       <c r="T27" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>2807</v>
+        <v>2806</v>
       </c>
       <c r="U27" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -9121,7 +9121,7 @@
       </c>
       <c r="AK27" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL27" s="4">
         <v>41640</v>
@@ -9215,7 +9215,7 @@
       </c>
       <c r="BP27" s="34">
         <f t="shared" ca="1" si="10"/>
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="BQ27" s="10" t="s">
         <v>120</v>
@@ -9228,7 +9228,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="28" spans="1:72" ht="14.25">
+    <row r="28" spans="1:72" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A28" s="26">
         <v>22</v>
       </c>
@@ -9286,11 +9286,11 @@
       </c>
       <c r="S28" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">45 Tahun 6 Bulan 28 Hari </v>
+        <v xml:space="preserve">45 Tahun 6 Bulan 29 Hari </v>
       </c>
       <c r="T28" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>3809</v>
+        <v>3808</v>
       </c>
       <c r="U28" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -9345,7 +9345,7 @@
       </c>
       <c r="AK28" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL28" s="4">
         <v>41640</v>
@@ -9441,7 +9441,7 @@
       </c>
       <c r="BP28" s="34">
         <f t="shared" ca="1" si="10"/>
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="BQ28" s="10" t="s">
         <v>120</v>
@@ -9454,7 +9454,7 @@
         <v>448</v>
       </c>
     </row>
-    <row r="29" spans="1:72" ht="14.25">
+    <row r="29" spans="1:72" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A29" s="26">
         <v>23</v>
       </c>
@@ -9512,11 +9512,11 @@
       </c>
       <c r="S29" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">50 Tahun 1 Bulan 30 Hari </v>
+        <v xml:space="preserve">50 Tahun 2 Bulan 0 Hari </v>
       </c>
       <c r="T29" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>2132</v>
+        <v>2131</v>
       </c>
       <c r="U29" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -9571,7 +9571,7 @@
       </c>
       <c r="AK29" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL29" s="4">
         <v>41640</v>
@@ -9667,7 +9667,7 @@
       </c>
       <c r="BP29" s="34">
         <f t="shared" ca="1" si="10"/>
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="BQ29" s="10" t="s">
         <v>120</v>
@@ -9680,7 +9680,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="30" spans="1:72" ht="14.25">
+    <row r="30" spans="1:72" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A30" s="26">
         <v>24</v>
       </c>
@@ -9738,11 +9738,11 @@
       </c>
       <c r="S30" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">30 Tahun 2 Bulan 2 Hari </v>
+        <v xml:space="preserve">30 Tahun 2 Bulan 3 Hari </v>
       </c>
       <c r="T30" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>9434</v>
+        <v>9433</v>
       </c>
       <c r="U30" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -9797,7 +9797,7 @@
       </c>
       <c r="AK30" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL30" s="4">
         <v>41640</v>
@@ -9893,7 +9893,7 @@
       </c>
       <c r="BP30" s="34">
         <f t="shared" ca="1" si="10"/>
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="BQ30" s="10" t="s">
         <v>120</v>
@@ -9906,7 +9906,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="31" spans="1:72" ht="14.25">
+    <row r="31" spans="1:72" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A31" s="26">
         <v>25</v>
       </c>
@@ -9964,11 +9964,11 @@
       </c>
       <c r="S31" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">36 Tahun 3 Bulan 22 Hari </v>
+        <v xml:space="preserve">36 Tahun 3 Bulan 23 Hari </v>
       </c>
       <c r="T31" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>7192</v>
+        <v>7191</v>
       </c>
       <c r="U31" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -10023,7 +10023,7 @@
       </c>
       <c r="AK31" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL31" s="4">
         <v>41640</v>
@@ -10119,7 +10119,7 @@
       </c>
       <c r="BP31" s="34">
         <f t="shared" ca="1" si="10"/>
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="BQ31" s="10" t="s">
         <v>120</v>
@@ -10132,7 +10132,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="32" spans="1:72" ht="14.25">
+    <row r="32" spans="1:72" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A32" s="26">
         <v>26</v>
       </c>
@@ -10190,11 +10190,11 @@
       </c>
       <c r="S32" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">33 Tahun 4 Bulan 17 Hari </v>
+        <v xml:space="preserve">33 Tahun 4 Bulan 18 Hari </v>
       </c>
       <c r="T32" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>8262</v>
+        <v>8261</v>
       </c>
       <c r="U32" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -10249,7 +10249,7 @@
       </c>
       <c r="AK32" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL32" s="4">
         <v>41640</v>
@@ -10345,7 +10345,7 @@
       </c>
       <c r="BP32" s="34">
         <f t="shared" ca="1" si="10"/>
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="BQ32" s="10" t="s">
         <v>120</v>
@@ -10358,7 +10358,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="33" spans="1:72" ht="14.25">
+    <row r="33" spans="1:72" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A33" s="26">
         <v>27</v>
       </c>
@@ -10416,11 +10416,11 @@
       </c>
       <c r="S33" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">49 Tahun 6 Bulan 1 Hari </v>
+        <v xml:space="preserve">49 Tahun 6 Bulan 2 Hari </v>
       </c>
       <c r="T33" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>2375</v>
+        <v>2374</v>
       </c>
       <c r="U33" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -10475,7 +10475,7 @@
       </c>
       <c r="AK33" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL33" s="4">
         <v>41640</v>
@@ -10569,7 +10569,7 @@
       </c>
       <c r="BP33" s="34">
         <f t="shared" ca="1" si="10"/>
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="BQ33" s="10" t="s">
         <v>120</v>
@@ -10582,7 +10582,7 @@
         <v>539</v>
       </c>
     </row>
-    <row r="34" spans="1:72" ht="14.25">
+    <row r="34" spans="1:72" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A34" s="26">
         <v>28</v>
       </c>
@@ -10640,11 +10640,11 @@
       </c>
       <c r="S34" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">44 Tahun 7 Bulan 22 Hari </v>
+        <v xml:space="preserve">44 Tahun 7 Bulan 23 Hari </v>
       </c>
       <c r="T34" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>4149</v>
+        <v>4148</v>
       </c>
       <c r="U34" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -10699,7 +10699,7 @@
       </c>
       <c r="AK34" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL34" s="4">
         <v>41640</v>
@@ -10795,7 +10795,7 @@
       </c>
       <c r="BP34" s="34">
         <f t="shared" ca="1" si="10"/>
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="BQ34" s="10" t="s">
         <v>120</v>
@@ -10808,7 +10808,7 @@
         <v>553</v>
       </c>
     </row>
-    <row r="35" spans="1:72" ht="14.25">
+    <row r="35" spans="1:72" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A35" s="26">
         <v>29</v>
       </c>
@@ -10866,11 +10866,11 @@
       </c>
       <c r="S35" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">29 Tahun 2 Bulan 2 Hari </v>
+        <v xml:space="preserve">29 Tahun 2 Bulan 3 Hari </v>
       </c>
       <c r="T35" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>9799</v>
+        <v>9798</v>
       </c>
       <c r="U35" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -10925,7 +10925,7 @@
       </c>
       <c r="AK35" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL35" s="4">
         <v>41640</v>
@@ -11019,7 +11019,7 @@
       </c>
       <c r="BP35" s="34">
         <f t="shared" ca="1" si="10"/>
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="BQ35" s="10" t="s">
         <v>120</v>
@@ -11032,7 +11032,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="36" spans="1:72" ht="14.25">
+    <row r="36" spans="1:72" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A36" s="26">
         <v>30</v>
       </c>
@@ -11090,11 +11090,11 @@
       </c>
       <c r="S36" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">28 Tahun 11 Bulan 28 Hari </v>
+        <v xml:space="preserve">28 Tahun 11 Bulan 29 Hari </v>
       </c>
       <c r="T36" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>9865</v>
+        <v>9864</v>
       </c>
       <c r="U36" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -11149,7 +11149,7 @@
       </c>
       <c r="AK36" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL36" s="4">
         <v>41640</v>
@@ -11243,7 +11243,7 @@
       </c>
       <c r="BP36" s="34">
         <f t="shared" ca="1" si="10"/>
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="BQ36" s="10" t="s">
         <v>120</v>
@@ -11256,7 +11256,7 @@
         <v>582</v>
       </c>
     </row>
-    <row r="37" spans="1:72" ht="14.25">
+    <row r="37" spans="1:72" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A37" s="26">
         <v>31</v>
       </c>
@@ -11314,11 +11314,11 @@
       </c>
       <c r="S37" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">54 Tahun 7 Bulan 22 Hari </v>
+        <v xml:space="preserve">54 Tahun 7 Bulan 23 Hari </v>
       </c>
       <c r="T37" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="U37" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -11373,7 +11373,7 @@
       </c>
       <c r="AK37" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL37" s="4">
         <v>41640</v>
@@ -11467,7 +11467,7 @@
       </c>
       <c r="BP37" s="34">
         <f t="shared" ca="1" si="10"/>
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="BQ37" s="10" t="s">
         <v>120</v>
@@ -11480,7 +11480,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="38" spans="1:72" ht="14.25">
+    <row r="38" spans="1:72" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A38" s="26">
         <v>32</v>
       </c>
@@ -11538,11 +11538,11 @@
       </c>
       <c r="S38" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">54 Tahun 0 Bulan 17 Hari </v>
+        <v xml:space="preserve">54 Tahun 0 Bulan 18 Hari </v>
       </c>
       <c r="T38" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="U38" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -11597,7 +11597,7 @@
       </c>
       <c r="AK38" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL38" s="4">
         <v>41640</v>
@@ -11693,7 +11693,7 @@
       </c>
       <c r="BP38" s="34">
         <f t="shared" ca="1" si="10"/>
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="BQ38" s="10" t="s">
         <v>120</v>
@@ -11706,7 +11706,7 @@
         <v>610</v>
       </c>
     </row>
-    <row r="39" spans="1:72" ht="14.25">
+    <row r="39" spans="1:72" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A39" s="26">
         <v>33</v>
       </c>
@@ -11764,11 +11764,11 @@
       </c>
       <c r="S39" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">41 Tahun 11 Bulan 26 Hari </v>
+        <v xml:space="preserve">41 Tahun 11 Bulan 27 Hari </v>
       </c>
       <c r="T39" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>5119</v>
+        <v>5118</v>
       </c>
       <c r="U39" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -11823,7 +11823,7 @@
       </c>
       <c r="AK39" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL39" s="4">
         <v>41640</v>
@@ -11917,7 +11917,7 @@
       </c>
       <c r="BP39" s="34">
         <f t="shared" ca="1" si="10"/>
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="BQ39" s="10" t="s">
         <v>120</v>
@@ -11930,7 +11930,7 @@
         <v>624</v>
       </c>
     </row>
-    <row r="40" spans="1:72" ht="14.25">
+    <row r="40" spans="1:72" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A40" s="26">
         <v>34</v>
       </c>
@@ -11988,11 +11988,11 @@
       </c>
       <c r="S40" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">34 Tahun 4 Bulan 15 Hari </v>
+        <v xml:space="preserve">34 Tahun 4 Bulan 16 Hari </v>
       </c>
       <c r="T40" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>7899</v>
+        <v>7898</v>
       </c>
       <c r="U40" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -12047,7 +12047,7 @@
       </c>
       <c r="AK40" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL40" s="4">
         <v>41640</v>
@@ -12143,7 +12143,7 @@
       </c>
       <c r="BP40" s="34">
         <f t="shared" ca="1" si="10"/>
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="BQ40" s="10" t="s">
         <v>120</v>
@@ -12156,7 +12156,7 @@
         <v>639</v>
       </c>
     </row>
-    <row r="41" spans="1:72" ht="14.25">
+    <row r="41" spans="1:72" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A41" s="26">
         <v>35</v>
       </c>
@@ -12214,11 +12214,11 @@
       </c>
       <c r="S41" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">33 Tahun 7 Bulan 15 Hari </v>
+        <v xml:space="preserve">33 Tahun 7 Bulan 16 Hari </v>
       </c>
       <c r="T41" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>8174</v>
+        <v>8173</v>
       </c>
       <c r="U41" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -12273,7 +12273,7 @@
       </c>
       <c r="AK41" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL41" s="4">
         <v>41640</v>
@@ -12367,7 +12367,7 @@
       </c>
       <c r="BP41" s="34">
         <f t="shared" ca="1" si="10"/>
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="BQ41" s="10" t="s">
         <v>120</v>
@@ -12380,7 +12380,7 @@
         <v>655</v>
       </c>
     </row>
-    <row r="42" spans="1:72" ht="14.25">
+    <row r="42" spans="1:72" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A42" s="26">
         <v>36</v>
       </c>
@@ -12438,11 +12438,11 @@
       </c>
       <c r="S42" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">35 Tahun 7 Bulan 30 Hari </v>
+        <v xml:space="preserve">35 Tahun 8 Bulan 0 Hari </v>
       </c>
       <c r="T42" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>7428</v>
+        <v>7427</v>
       </c>
       <c r="U42" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -12497,7 +12497,7 @@
       </c>
       <c r="AK42" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL42" s="4">
         <v>41640</v>
@@ -12591,7 +12591,7 @@
       </c>
       <c r="BP42" s="34">
         <f t="shared" ca="1" si="10"/>
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="BQ42" s="10" t="s">
         <v>120</v>
@@ -12604,7 +12604,7 @@
         <v>667</v>
       </c>
     </row>
-    <row r="43" spans="1:72" ht="14.25">
+    <row r="43" spans="1:72" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A43" s="26">
         <v>37</v>
       </c>
@@ -12662,11 +12662,11 @@
       </c>
       <c r="S43" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">37 Tahun 0 Bulan 19 Hari </v>
+        <v xml:space="preserve">37 Tahun 0 Bulan 20 Hari </v>
       </c>
       <c r="T43" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>6921</v>
+        <v>6920</v>
       </c>
       <c r="U43" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -12721,7 +12721,7 @@
       </c>
       <c r="AK43" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL43" s="4">
         <v>41640</v>
@@ -12817,7 +12817,7 @@
       </c>
       <c r="BP43" s="34">
         <f t="shared" ca="1" si="10"/>
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="BQ43" s="10" t="s">
         <v>120</v>
@@ -12830,7 +12830,7 @@
         <v>679</v>
       </c>
     </row>
-    <row r="44" spans="1:72" ht="14.25">
+    <row r="44" spans="1:72" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A44" s="26">
         <v>38</v>
       </c>
@@ -12888,11 +12888,11 @@
       </c>
       <c r="S44" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">50 Tahun 7 Bulan 19 Hari </v>
+        <v xml:space="preserve">50 Tahun 7 Bulan 20 Hari </v>
       </c>
       <c r="T44" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>1960</v>
+        <v>1959</v>
       </c>
       <c r="U44" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -12947,7 +12947,7 @@
       </c>
       <c r="AK44" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL44" s="4">
         <v>41640</v>
@@ -13041,7 +13041,7 @@
       </c>
       <c r="BP44" s="34">
         <f t="shared" ca="1" si="10"/>
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="BQ44" s="10" t="s">
         <v>120</v>
@@ -13054,7 +13054,7 @@
         <v>693</v>
       </c>
     </row>
-    <row r="45" spans="1:72" ht="14.25">
+    <row r="45" spans="1:72" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A45" s="26">
         <v>39</v>
       </c>
@@ -13112,11 +13112,11 @@
       </c>
       <c r="S45" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">50 Tahun 5 Bulan 16 Hari </v>
+        <v xml:space="preserve">50 Tahun 5 Bulan 17 Hari </v>
       </c>
       <c r="T45" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="U45" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -13171,7 +13171,7 @@
       </c>
       <c r="AK45" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL45" s="4">
         <v>41640</v>
@@ -13265,7 +13265,7 @@
       </c>
       <c r="BP45" s="34">
         <f t="shared" ca="1" si="10"/>
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="BQ45" s="10" t="s">
         <v>120</v>
@@ -13278,7 +13278,7 @@
         <v>706</v>
       </c>
     </row>
-    <row r="46" spans="1:72" ht="14.25">
+    <row r="46" spans="1:72" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A46" s="26">
         <v>40</v>
       </c>
@@ -13336,11 +13336,11 @@
       </c>
       <c r="S46" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">35 Tahun 11 Bulan 6 Hari </v>
+        <v xml:space="preserve">35 Tahun 11 Bulan 7 Hari </v>
       </c>
       <c r="T46" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>7330</v>
+        <v>7329</v>
       </c>
       <c r="U46" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -13395,7 +13395,7 @@
       </c>
       <c r="AK46" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL46" s="4">
         <v>41640</v>
@@ -13491,7 +13491,7 @@
       </c>
       <c r="BP46" s="34">
         <f t="shared" ca="1" si="10"/>
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="BQ46" s="10" t="s">
         <v>120</v>
@@ -13504,7 +13504,7 @@
         <v>719</v>
       </c>
     </row>
-    <row r="47" spans="1:72" ht="14.25">
+    <row r="47" spans="1:72" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A47" s="26">
         <v>41</v>
       </c>
@@ -13562,11 +13562,11 @@
       </c>
       <c r="S47" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">30 Tahun 4 Bulan 24 Hari </v>
+        <v xml:space="preserve">30 Tahun 4 Bulan 25 Hari </v>
       </c>
       <c r="T47" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>9351</v>
+        <v>9350</v>
       </c>
       <c r="U47" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -13621,7 +13621,7 @@
       </c>
       <c r="AK47" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL47" s="4">
         <v>41640</v>
@@ -13715,7 +13715,7 @@
       </c>
       <c r="BP47" s="34">
         <f t="shared" ca="1" si="10"/>
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="BQ47" s="10" t="s">
         <v>120</v>
@@ -13728,7 +13728,7 @@
         <v>734</v>
       </c>
     </row>
-    <row r="48" spans="1:72" ht="14.25">
+    <row r="48" spans="1:72" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A48" s="26">
         <v>42</v>
       </c>
@@ -13786,11 +13786,11 @@
       </c>
       <c r="S48" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">40 Tahun 6 Bulan 18 Hari </v>
+        <v xml:space="preserve">40 Tahun 6 Bulan 19 Hari </v>
       </c>
       <c r="T48" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>5645</v>
+        <v>5644</v>
       </c>
       <c r="U48" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -13845,7 +13845,7 @@
       </c>
       <c r="AK48" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL48" s="4">
         <v>41640</v>
@@ -13939,7 +13939,7 @@
       </c>
       <c r="BP48" s="34">
         <f t="shared" ca="1" si="10"/>
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="BQ48" s="10" t="s">
         <v>120</v>
@@ -13952,7 +13952,7 @@
         <v>748</v>
       </c>
     </row>
-    <row r="49" spans="1:72" ht="14.25">
+    <row r="49" spans="1:72" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A49" s="26">
         <v>43</v>
       </c>
@@ -14010,11 +14010,11 @@
       </c>
       <c r="S49" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">35 Tahun 11 Bulan 20 Hari </v>
+        <v xml:space="preserve">35 Tahun 11 Bulan 21 Hari </v>
       </c>
       <c r="T49" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>7316</v>
+        <v>7315</v>
       </c>
       <c r="U49" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -14069,7 +14069,7 @@
       </c>
       <c r="AK49" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL49" s="4">
         <v>41640</v>
@@ -14165,7 +14165,7 @@
       </c>
       <c r="BP49" s="34">
         <f t="shared" ca="1" si="10"/>
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="BQ49" s="10" t="s">
         <v>120</v>
@@ -14178,7 +14178,7 @@
         <v>763</v>
       </c>
     </row>
-    <row r="50" spans="1:72" ht="14.25">
+    <row r="50" spans="1:72" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A50" s="26">
         <v>44</v>
       </c>
@@ -14236,11 +14236,11 @@
       </c>
       <c r="S50" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">45 Tahun 2 Bulan 19 Hari </v>
+        <v xml:space="preserve">45 Tahun 2 Bulan 20 Hari </v>
       </c>
       <c r="T50" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>3938</v>
+        <v>3937</v>
       </c>
       <c r="U50" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -14295,7 +14295,7 @@
       </c>
       <c r="AK50" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL50" s="4">
         <v>41640</v>
@@ -14389,7 +14389,7 @@
       </c>
       <c r="BP50" s="34">
         <f t="shared" ca="1" si="10"/>
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="BQ50" s="10" t="s">
         <v>120</v>
@@ -14402,7 +14402,7 @@
         <v>776</v>
       </c>
     </row>
-    <row r="51" spans="1:72" ht="14.25">
+    <row r="51" spans="1:72" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A51" s="26">
         <v>45</v>
       </c>
@@ -14460,11 +14460,11 @@
       </c>
       <c r="S51" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">34 Tahun 4 Bulan 27 Hari </v>
+        <v xml:space="preserve">34 Tahun 4 Bulan 28 Hari </v>
       </c>
       <c r="T51" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>7887</v>
+        <v>7886</v>
       </c>
       <c r="U51" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -14519,7 +14519,7 @@
       </c>
       <c r="AK51" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL51" s="4">
         <v>41640</v>
@@ -14613,7 +14613,7 @@
       </c>
       <c r="BP51" s="34">
         <f t="shared" ca="1" si="10"/>
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="BQ51" s="10" t="s">
         <v>120</v>
@@ -14626,7 +14626,7 @@
         <v>789</v>
       </c>
     </row>
-    <row r="52" spans="1:72" ht="14.25">
+    <row r="52" spans="1:72" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A52" s="26">
         <v>46</v>
       </c>
@@ -14684,11 +14684,11 @@
       </c>
       <c r="S52" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">31 Tahun 2 Bulan 11 Hari </v>
+        <v xml:space="preserve">31 Tahun 2 Bulan 12 Hari </v>
       </c>
       <c r="T52" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>9059</v>
+        <v>9058</v>
       </c>
       <c r="U52" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -14743,7 +14743,7 @@
       </c>
       <c r="AK52" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL52" s="4">
         <v>41640</v>
@@ -14837,7 +14837,7 @@
       </c>
       <c r="BP52" s="34">
         <f t="shared" ca="1" si="10"/>
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="BQ52" s="10" t="s">
         <v>120</v>
@@ -14850,7 +14850,7 @@
         <v>804</v>
       </c>
     </row>
-    <row r="53" spans="1:72" ht="14.25">
+    <row r="53" spans="1:72" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A53" s="26">
         <v>47</v>
       </c>
@@ -14908,11 +14908,11 @@
       </c>
       <c r="S53" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">29 Tahun 7 Bulan 9 Hari </v>
+        <v xml:space="preserve">29 Tahun 7 Bulan 10 Hari </v>
       </c>
       <c r="T53" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>9641</v>
+        <v>9640</v>
       </c>
       <c r="U53" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -14965,7 +14965,7 @@
       </c>
       <c r="AK53" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL53" s="4">
         <v>46144</v>
@@ -15059,7 +15059,7 @@
       </c>
       <c r="BP53" s="34">
         <f t="shared" ca="1" si="10"/>
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="BQ53" s="10" t="s">
         <v>120</v>
@@ -15072,7 +15072,7 @@
         <v>817</v>
       </c>
     </row>
-    <row r="54" spans="1:72" ht="14.25">
+    <row r="54" spans="1:72" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A54" s="26">
         <v>48</v>
       </c>
@@ -15130,11 +15130,11 @@
       </c>
       <c r="S54" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">33 Tahun 10 Bulan 24 Hari </v>
+        <v xml:space="preserve">33 Tahun 10 Bulan 25 Hari </v>
       </c>
       <c r="T54" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>8074</v>
+        <v>8073</v>
       </c>
       <c r="U54" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -15189,7 +15189,7 @@
       </c>
       <c r="AK54" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL54" s="4">
         <v>41640</v>
@@ -15285,7 +15285,7 @@
       </c>
       <c r="BP54" s="34">
         <f t="shared" ca="1" si="10"/>
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="BQ54" s="10" t="s">
         <v>120</v>
@@ -15298,7 +15298,7 @@
         <v>835</v>
       </c>
     </row>
-    <row r="55" spans="1:72" ht="14.25">
+    <row r="55" spans="1:72" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A55" s="26">
         <v>49</v>
       </c>
@@ -15356,11 +15356,11 @@
       </c>
       <c r="S55" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">39 Tahun 2 Bulan 22 Hari </v>
+        <v xml:space="preserve">39 Tahun 2 Bulan 23 Hari </v>
       </c>
       <c r="T55" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>6126</v>
+        <v>6125</v>
       </c>
       <c r="U55" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -15415,7 +15415,7 @@
       </c>
       <c r="AK55" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL55" s="4">
         <v>41640</v>
@@ -15511,7 +15511,7 @@
       </c>
       <c r="BP55" s="34">
         <f t="shared" ca="1" si="10"/>
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="BQ55" s="10" t="s">
         <v>120</v>
@@ -15524,7 +15524,7 @@
         <v>854</v>
       </c>
     </row>
-    <row r="56" spans="1:72" ht="14.25">
+    <row r="56" spans="1:72" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A56" s="26">
         <v>50</v>
       </c>
@@ -15582,11 +15582,11 @@
       </c>
       <c r="S56" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">33 Tahun 6 Bulan 14 Hari </v>
+        <v xml:space="preserve">33 Tahun 6 Bulan 15 Hari </v>
       </c>
       <c r="T56" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>8206</v>
+        <v>8205</v>
       </c>
       <c r="U56" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -15641,7 +15641,7 @@
       </c>
       <c r="AK56" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL56" s="4">
         <v>41640</v>
@@ -15737,7 +15737,7 @@
       </c>
       <c r="BP56" s="34">
         <f t="shared" ca="1" si="10"/>
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="BQ56" s="10" t="s">
         <v>120</v>
@@ -15750,7 +15750,7 @@
         <v>871</v>
       </c>
     </row>
-    <row r="57" spans="1:72" ht="14.25">
+    <row r="57" spans="1:72" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A57" s="26">
         <v>51</v>
       </c>
@@ -15808,11 +15808,11 @@
       </c>
       <c r="S57" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">33 Tahun 3 Bulan 17 Hari </v>
+        <v xml:space="preserve">33 Tahun 3 Bulan 18 Hari </v>
       </c>
       <c r="T57" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>8293</v>
+        <v>8292</v>
       </c>
       <c r="U57" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -15867,7 +15867,7 @@
       </c>
       <c r="AK57" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL57" s="4">
         <v>41640</v>
@@ -15963,7 +15963,7 @@
       </c>
       <c r="BP57" s="34">
         <f t="shared" ca="1" si="10"/>
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="BQ57" s="10" t="s">
         <v>120</v>
@@ -15976,7 +15976,7 @@
         <v>890</v>
       </c>
     </row>
-    <row r="58" spans="1:72" ht="14.25">
+    <row r="58" spans="1:72" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A58" s="26">
         <v>52</v>
       </c>
@@ -16034,11 +16034,11 @@
       </c>
       <c r="S58" s="31" t="str">
         <f t="shared" ca="1" si="7"/>
-        <v xml:space="preserve">29 Tahun 5 Bulan 7 Hari </v>
+        <v xml:space="preserve">29 Tahun 5 Bulan 8 Hari </v>
       </c>
       <c r="T58" s="32">
         <f t="shared" ca="1" si="3"/>
-        <v>9705</v>
+        <v>9704</v>
       </c>
       <c r="U58" s="30" t="str">
         <f t="shared" ca="1" si="4"/>
@@ -16093,7 +16093,7 @@
       </c>
       <c r="AK58" s="34">
         <f t="shared" ca="1" si="8"/>
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="AL58" s="4">
         <v>41640</v>
@@ -16189,7 +16189,7 @@
       </c>
       <c r="BP58" s="50">
         <f t="shared" ca="1" si="10"/>
-        <v>-159</v>
+        <v>-160</v>
       </c>
       <c r="BQ58" s="10" t="s">
         <v>120</v>
@@ -16202,7 +16202,7 @@
         <v>899</v>
       </c>
     </row>
-    <row r="59" spans="1:72" ht="13.15">
+    <row r="59" spans="1:72" ht="13.15" x14ac:dyDescent="0.4">
       <c r="A59" s="44"/>
       <c r="B59" s="52"/>
       <c r="C59" s="52"/>
@@ -16279,7 +16279,7 @@
       <c r="BS59" s="44"/>
       <c r="BT59" s="44"/>
     </row>
-    <row r="60" spans="1:72" ht="13.15">
+    <row r="60" spans="1:72" ht="13.15" x14ac:dyDescent="0.4">
       <c r="A60" s="44"/>
       <c r="B60" s="52"/>
       <c r="C60" s="52"/>
@@ -16360,7 +16360,7 @@
       <c r="BS60" s="44"/>
       <c r="BT60" s="44"/>
     </row>
-    <row r="61" spans="1:72">
+    <row r="61" spans="1:72" x14ac:dyDescent="0.35">
       <c r="A61" s="44"/>
       <c r="B61" s="52"/>
       <c r="C61" s="52"/>

</xml_diff>